<commit_message>
punch confirmation form updated
</commit_message>
<xml_diff>
--- a/uploads/excel/Apartment_Import_Template.xlsx
+++ b/uploads/excel/Apartment_Import_Template.xlsx
@@ -459,7 +459,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:X2"/>
+  <dimension ref="A1:W2"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -470,21 +470,20 @@
     <col min="7" max="7" width="20.83203125" customWidth="1"/>
     <col min="8" max="8" width="25.83203125" customWidth="1"/>
     <col min="9" max="9" width="35.83203125" customWidth="1"/>
-    <col min="10" max="10" width="25.83203125" customWidth="1"/>
+    <col min="10" max="10" width="22.83203125" customWidth="1"/>
     <col min="11" max="11" width="22.83203125" customWidth="1"/>
-    <col min="12" max="12" width="22.83203125" customWidth="1"/>
-    <col min="13" max="13" width="30.83203125" customWidth="1"/>
+    <col min="12" max="12" width="30.83203125" customWidth="1"/>
+    <col min="13" max="13" width="15.83203125" customWidth="1"/>
     <col min="14" max="14" width="15.83203125" customWidth="1"/>
-    <col min="15" max="15" width="15.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="20.83203125" customWidth="1"/>
-    <col min="18" max="18" width="18.83203125" customWidth="1"/>
-    <col min="19" max="19" width="22.83203125" customWidth="1"/>
-    <col min="20" max="20" width="28.83203125" customWidth="1"/>
-    <col min="21" max="21" width="32.83203125" customWidth="1"/>
-    <col min="22" max="22" width="25.83203125" customWidth="1"/>
-    <col min="23" max="23" width="18.83203125" customWidth="1"/>
-    <col min="24" max="24" width="12.83203125" customWidth="1"/>
+    <col min="15" max="15" width="18.83203125" customWidth="1"/>
+    <col min="16" max="16" width="20.83203125" customWidth="1"/>
+    <col min="17" max="17" width="18.83203125" customWidth="1"/>
+    <col min="18" max="18" width="22.83203125" customWidth="1"/>
+    <col min="19" max="19" width="28.83203125" customWidth="1"/>
+    <col min="20" max="20" width="32.83203125" customWidth="1"/>
+    <col min="21" max="21" width="25.83203125" customWidth="1"/>
+    <col min="22" max="22" width="18.83203125" customWidth="1"/>
+    <col min="23" max="23" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
@@ -516,48 +515,45 @@
         <v>email</v>
       </c>
       <c r="J1" s="3" t="str">
-        <v>profile_photo</v>
+        <v>aadhaar_number</v>
       </c>
       <c r="K1" s="3" t="str">
-        <v>aadhaar_number</v>
+        <v>occupation</v>
       </c>
       <c r="L1" s="3" t="str">
-        <v>occupation</v>
+        <v>apartment_name</v>
       </c>
       <c r="M1" s="3" t="str">
-        <v>apartment_name</v>
+        <v>block_tower</v>
       </c>
       <c r="N1" s="3" t="str">
-        <v>block_tower</v>
+        <v>floor_number</v>
       </c>
       <c r="O1" s="3" t="str">
-        <v>floor_number</v>
+        <v>flat_number</v>
       </c>
       <c r="P1" s="3" t="str">
-        <v>flat_number</v>
+        <v>ownership_type</v>
       </c>
       <c r="Q1" s="3" t="str">
-        <v>ownership_type</v>
+        <v>move_in_date</v>
       </c>
       <c r="R1" s="3" t="str">
-        <v>move_in_date</v>
+        <v>family_member_count</v>
       </c>
       <c r="S1" s="3" t="str">
-        <v>family_member_count</v>
+        <v>emergency_contact_name</v>
       </c>
       <c r="T1" s="3" t="str">
-        <v>emergency_contact_name</v>
+        <v>emergency_contact_relationship</v>
       </c>
       <c r="U1" s="3" t="str">
-        <v>emergency_contact_relationship</v>
+        <v>emergency_contact_mobile</v>
       </c>
       <c r="V1" s="3" t="str">
-        <v>emergency_contact_mobile</v>
+        <v>member_type</v>
       </c>
       <c r="W1" s="3" t="str">
-        <v>member_type</v>
-      </c>
-      <c r="X1" s="3" t="str">
         <v>status</v>
       </c>
     </row>
@@ -590,54 +586,51 @@
         <v>john@test.com</v>
       </c>
       <c r="J2" s="4" t="str">
-        <v/>
+        <v>123456789012</v>
       </c>
       <c r="K2" s="4" t="str">
-        <v>123456789012</v>
+        <v>Engineer</v>
       </c>
       <c r="L2" s="4" t="str">
-        <v>Engineer</v>
+        <v>Green Residency</v>
       </c>
       <c r="M2" s="4" t="str">
-        <v>Green Residency</v>
-      </c>
-      <c r="N2" s="4" t="str">
         <v>A</v>
       </c>
-      <c r="O2" s="4">
+      <c r="N2" s="4">
         <v>2</v>
       </c>
+      <c r="O2" s="4" t="str">
+        <v>201</v>
+      </c>
       <c r="P2" s="4" t="str">
-        <v>201</v>
+        <v>OWNER</v>
       </c>
       <c r="Q2" s="4" t="str">
-        <v>OWNER</v>
-      </c>
-      <c r="R2" s="4" t="str">
         <v>2025-01-01</v>
       </c>
-      <c r="S2" s="4">
+      <c r="R2" s="4">
         <v>2</v>
       </c>
+      <c r="S2" s="4" t="str">
+        <v>Mary</v>
+      </c>
       <c r="T2" s="4" t="str">
-        <v>Mary</v>
+        <v>WIFE</v>
       </c>
       <c r="U2" s="4" t="str">
-        <v>WIFE</v>
+        <v>9876543211</v>
       </c>
       <c r="V2" s="4" t="str">
-        <v>9876543211</v>
-      </c>
-      <c r="W2" s="4" t="str">
         <v>RESIDENT</v>
       </c>
-      <c r="X2" s="4" t="b">
+      <c r="W2" s="4" t="b">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:X2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -655,21 +648,20 @@
     <col min="7" max="7" width="20.83203125" customWidth="1"/>
     <col min="8" max="8" width="25.83203125" customWidth="1"/>
     <col min="9" max="9" width="35.83203125" customWidth="1"/>
-    <col min="10" max="10" width="25.83203125" customWidth="1"/>
+    <col min="10" max="10" width="22.83203125" customWidth="1"/>
     <col min="11" max="11" width="22.83203125" customWidth="1"/>
-    <col min="12" max="12" width="22.83203125" customWidth="1"/>
-    <col min="13" max="13" width="30.83203125" customWidth="1"/>
+    <col min="12" max="12" width="30.83203125" customWidth="1"/>
+    <col min="13" max="13" width="15.83203125" customWidth="1"/>
     <col min="14" max="14" width="15.83203125" customWidth="1"/>
-    <col min="15" max="15" width="15.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="20.83203125" customWidth="1"/>
-    <col min="18" max="18" width="18.83203125" customWidth="1"/>
-    <col min="19" max="19" width="22.83203125" customWidth="1"/>
-    <col min="20" max="20" width="28.83203125" customWidth="1"/>
-    <col min="21" max="21" width="32.83203125" customWidth="1"/>
-    <col min="22" max="22" width="25.83203125" customWidth="1"/>
-    <col min="23" max="23" width="18.83203125" customWidth="1"/>
-    <col min="24" max="24" width="12.83203125" customWidth="1"/>
+    <col min="15" max="15" width="18.83203125" customWidth="1"/>
+    <col min="16" max="16" width="20.83203125" customWidth="1"/>
+    <col min="17" max="17" width="18.83203125" customWidth="1"/>
+    <col min="18" max="18" width="22.83203125" customWidth="1"/>
+    <col min="19" max="19" width="28.83203125" customWidth="1"/>
+    <col min="20" max="20" width="32.83203125" customWidth="1"/>
+    <col min="21" max="21" width="25.83203125" customWidth="1"/>
+    <col min="22" max="22" width="18.83203125" customWidth="1"/>
+    <col min="23" max="23" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
@@ -726,21 +718,20 @@
     <col min="7" max="7" width="20.83203125" customWidth="1"/>
     <col min="8" max="8" width="25.83203125" customWidth="1"/>
     <col min="9" max="9" width="35.83203125" customWidth="1"/>
-    <col min="10" max="10" width="25.83203125" customWidth="1"/>
+    <col min="10" max="10" width="22.83203125" customWidth="1"/>
     <col min="11" max="11" width="22.83203125" customWidth="1"/>
-    <col min="12" max="12" width="22.83203125" customWidth="1"/>
-    <col min="13" max="13" width="30.83203125" customWidth="1"/>
+    <col min="12" max="12" width="30.83203125" customWidth="1"/>
+    <col min="13" max="13" width="15.83203125" customWidth="1"/>
     <col min="14" max="14" width="15.83203125" customWidth="1"/>
-    <col min="15" max="15" width="15.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="20.83203125" customWidth="1"/>
-    <col min="18" max="18" width="18.83203125" customWidth="1"/>
-    <col min="19" max="19" width="22.83203125" customWidth="1"/>
-    <col min="20" max="20" width="28.83203125" customWidth="1"/>
-    <col min="21" max="21" width="32.83203125" customWidth="1"/>
-    <col min="22" max="22" width="25.83203125" customWidth="1"/>
-    <col min="23" max="23" width="18.83203125" customWidth="1"/>
-    <col min="24" max="24" width="12.83203125" customWidth="1"/>
+    <col min="15" max="15" width="18.83203125" customWidth="1"/>
+    <col min="16" max="16" width="20.83203125" customWidth="1"/>
+    <col min="17" max="17" width="18.83203125" customWidth="1"/>
+    <col min="18" max="18" width="22.83203125" customWidth="1"/>
+    <col min="19" max="19" width="28.83203125" customWidth="1"/>
+    <col min="20" max="20" width="32.83203125" customWidth="1"/>
+    <col min="21" max="21" width="25.83203125" customWidth="1"/>
+    <col min="22" max="22" width="18.83203125" customWidth="1"/>
+    <col min="23" max="23" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">

</xml_diff>